<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.003-05 La feuille qui danse
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.003-05.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.003-05.xlsx
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nino veut garder une feuille qui danse dans son seau vert. Elle s'envole. Il reprend seau, manteau et ours pour lui faire une place près de la feuille de la fenêtre.</t>
+          <t>Nino connaît le toc de la fenêtre. Un éclat de vitre cligne sur le verre. Il veut une feuille dans le seau vert, maintenant. Il plaque trop vite : la feuille s'envole, manche tordue, ours au toboggan. Il reprend seau, manteau, ours. Merci vécu. À la maison il veut glisser trop fort. Il refuse de foncer, retrouve l'éclat, pose le seau. La feuille tapote.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une feuille collée à la vitre tapote. Toc, toc. Le soleil de l'après-midi la rend orange. Maman ouvre un peu la fenêtre. Un souffle d'air entre. Tu as vu la feuille, Nino ? Elle est orange. Elle veut rentrer. Maman la pose sur le rebord. On va à l'aire de jeux ? Oui, maman. Je veux une feuille, moi aussi. On regardera. Ils prennent le sac. La rue est calme. En ce moment, Nino est à l'aire de jeux. Le sable est un peu chaud. Maman s'assoit au bord. Nino a un seau vert. Il a un manteau bleu posé au bord. Il a son doudou ours. Le petit toboggan est tiède. Il est chaud, maman. Le soleil l'a touché. Nino verse le sable. Ça fait chh. Une feuille passe. Une feuille, maman ! Comme celle de la fenêtre. Elle danse. La feuille se pose dans le seau. Nino la sort tout doux. Elle habite ici. Le vent reprend la feuille. Elle s'envole au-dessus du bac. Elle est partie. Elle vole encore. C'est l'heure. La feuille aussi ? La feuille peut voler. Tes affaires viennent à la maison. On reprend ses affaires, avant de partir. Nino cherche le seau. Le seau est encore vert, un peu sableux. Il le prend. J'ai le seau. Bien. On lui fera une place, à la maison. Le manteau est au bord. Une manche est à l'envers. L'ours est près du toboggan.</t>
+          <t>Une ombre orange traverse le plancher, lente. Elle grimpe le mur, jusqu'au rebord. Derrière le verre, une feuille tapote. Toc, toc. Le soleil d'après-midi la rend orange. Maman ouvre un peu la fenêtre. Un souffle d'air entre, tiède. Tu as vu la feuille, Nino ? Elle danse ! Sur la vitre, un éclat de vitre cligne. Tu vois l'éclat ? Il brille, sur le verre. Maman pose la feuille sur le rebord. Je veux une feuille, maintenant ! Dans mon seau vert ! On va à l'aire de jeux. Ils prennent le sac, près de la porte. La rue sent le sable chaud. En ce moment, Nino pose le seau vert au bac. Le sable est tiède, un peu collant. Maman s'assoit au bord, à sa hauteur. Le bac du toboggan tiède sent le sable. Le manteau bleu attend au bord, plié. L'ours doudou s'appuie au petit toboggan. Le toboggan est chaud. Le soleil l'a touché. Nino verse le sable. Ça fait chh, dans le seau. Une feuille orange passe, basse. La mienne, maintenant ! Elle se pose dans le seau vert. Nino plaque la main dessus, vite. Le seau bascule. Du sable glisse, chaud. La feuille s'envole au-dessus du bac. Elle est partie ! Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Nino veut courir après la feuille. Il tire le seau et le manteau, ensemble. La manche se tord, à l'envers. L'ours bascule, près du toboggan. Ça reste coincé ! C'est l'heure. La feuille aussi ? La feuille peut voler. Toi, tu reprends le seau ? Nino cherche le seau. Le seau est vert, un peu sableux. Il le prend. J'ai le seau. Le manteau est au bord. Une manche est à l'envers. L'ours est près du toboggan. Tu poses le seau un moment ? Maman s'accroupit à sa hauteur. Tu regardes tes affaires ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une feuille collée à la vitre tapote. Toc, toc. Le soleil de l'après-midi la rend orange. Maman ouvre un peu la fenêtre. Un souffle d'air entre. Tu as vu la feuille, Nino ? Elle est orange. Elle veut rentrer. Maman la pose sur le rebord. On va à l'aire de jeux ? Oui, maman. Je veux une feuille, moi aussi. On regardera. Ils prennent le sac. La rue est calme. En ce moment, Nino est à l'aire de jeux. Le sable est un peu chaud. Maman s'assoit au bord. Nino a un seau vert. Il a un manteau bleu posé au bord. Il a son doudou ours. Le petit toboggan est tiède. Il est chaud, maman. Le soleil l'a touché. Nino verse le sable. Ça fait chh. Une feuille passe. Une feuille, maman ! Comme celle de la fenêtre. Elle danse. La feuille se pose dans le seau. Nino la sort tout doux. Elle habite ici. Le vent reprend la feuille. Elle s'envole au-dessus du bac. Elle est partie. Elle vole encore. C'est l'heure. La feuille aussi ? La feuille peut voler. Tes affaires viennent à la maison. On reprend ses affaires, avant de partir. Nino cherche le seau. Le seau est encore vert, un peu sableux. Il le prend. J'ai le seau. Bien. On lui fera une place, à la maison. Le manteau est au bord. Une manche est à l'envers. L'ours est près du toboggan.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une ombre orange traverse le plancher, lente. Elle grimpe le mur, jusqu'au rebord. Derrière le verre, une feuille tapote. Toc, toc. Le soleil d'après-midi la rend orange. Maman ouvre un peu la fenêtre. Un souffle d'air entre, tiède. Tu as vu la feuille, Nino ? Elle danse ! Sur la vitre, un &lt;emphasis level="moderate"&gt;éclat de vitre&lt;/emphasis&gt; cligne. Tu vois l'éclat ? Il brille, sur le verre. Maman pose la feuille sur le rebord. Je veux une feuille, maintenant ! Dans mon seau vert ! On va à l'aire de jeux. Ils prennent le sac, près de la porte. La rue sent le sable chaud. En ce moment, Nino pose le seau vert au bac. Le sable est tiède, un peu collant. Maman s'assoit au bord, à sa hauteur. Le bac du toboggan tiède sent le sable. Le manteau bleu attend au bord, plié. L'ours doudou s'appuie au petit toboggan. Le toboggan est chaud. Le soleil l'a touché. Nino verse le sable. Ça fait chh, dans le seau. Une feuille orange passe, basse. La mienne, maintenant ! Elle se pose dans le seau vert. Nino plaque la main dessus, vite. Le seau bascule. Du sable glisse, chaud. La feuille s'envole au-dessus du bac. Elle est partie ! Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Nino veut courir après la feuille. Il tire le seau et le manteau, ensemble. La manche se tord, à l'envers. L'ours bascule, près du toboggan. Ça reste coincé ! C'est l'heure. La feuille aussi ? La feuille peut voler. Toi, tu reprends le seau ? Nino cherche le seau. Le seau est vert, un peu sableux. Il le prend. J'ai le seau. Le manteau est au bord. Une manche est à l'envers. L'ours est près du toboggan. Tu poses le seau un moment ? Maman s'accroupit à sa hauteur. Tu regardes tes affaires ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Clément joue à l'aire de jeux, près de maman. Le sable est un peu chaud. Clément a un seau vert. Il a un manteau bleu posé au bord. Il a son doudou ours. Clément verse le sable. Ça fait chh. Une feuille passe. Maman dit : c'est l'heure. On va &lt;emphasis&gt;reprendre&lt;/emphasis&gt; ses affaires avant de partir. Clément cherche le seau. Il le prend. Clément cherche le manteau. Il le prend. Clément cherche le doudou. Il le prend. Ses affaires sont dans ses bras. Parce qu'il a repris ses affaires, on peut rentrer. Maman dit : merci Clément. C'était avant de partir. Ils marchent vers la maison. Le seau cogne un peu. Le doudou est contre lui. Maman reste à côté. [pause]</t>
+          <t>Une ombre orange traverse le plancher, lente. Elle grimpe le mur, jusqu'au rebord. Derrière le verre, une feuille tapote. Toc, toc. Le soleil d'après-midi la rend orange. Maman ouvre un peu la fenêtre. Un souffle d'air entre, tiède. Tu as vu la feuille, Nino ? Elle danse ! Sur la vitre, un &lt;emphasis&gt;éclat de vitre&lt;/emphasis&gt; cligne. Tu vois l'éclat ? Il brille, sur le verre. Maman pose la feuille sur le rebord. Je veux une feuille, maintenant ! Dans mon seau vert ! On va à l'aire de jeux. Ils prennent le sac, près de la porte. La rue sent le sable chaud. En ce moment, Nino pose le seau vert au bac. Le sable est tiède, un peu collant. Maman s'assoit au bord, à sa hauteur. Le bac du toboggan tiède sent le sable. Le manteau bleu attend au bord, plié. L'ours doudou s'appuie au petit toboggan. Le toboggan est chaud. Le soleil l'a touché. Nino verse le sable. Ça fait chh, dans le seau. Une feuille orange passe, basse. La mienne, maintenant ! Elle se pose dans le seau vert. Nino plaque la main dessus, vite. Le seau bascule. Du sable glisse, chaud. La feuille s'envole au-dessus du bac. Elle est partie ! Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Nino veut courir après la feuille. Il tire le seau et le manteau, ensemble. La manche se tord, à l'envers. L'ours bascule, près du toboggan. Ça reste coincé ! C'est l'heure. La feuille aussi ? La feuille peut voler. Toi, tu reprends le seau ? Nino cherche le seau. Le seau est vert, un peu sableux. Il le prend. J'ai le seau. Le manteau est au bord. Une manche est à l'envers. L'ours est près du toboggan. Tu poses le seau un moment ? Maman s'accroupit à sa hauteur. Tu regardes tes affaires ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>reprendre</t>
+          <t>éclat de vitre</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,65 +1326,75 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_feuille_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une feuille collée à la vitre tapote.
+          <t>narrateur|Une ombre orange traverse le plancher, lente.
+narrateur|Elle grimpe le mur, jusqu'au rebord.
+narrateur|Derrière le verre, une feuille tapote.
 narrateur|Toc, toc.
-narrateur|Le soleil de l'après-midi la rend orange.
+narrateur|Le soleil d'après-midi la rend orange.
 narrateur|Maman ouvre un peu la fenêtre.
-narrateur|Un souffle d'air entre.
+narrateur|Un souffle d'air entre, tiède.
 maman|Tu as vu la feuille, Nino ?
-enfant-m|Elle est orange.
-maman|Elle veut rentrer.
-narrateur|Maman la pose sur le rebord.
-maman|On va à l'aire de jeux ?
-enfant-m|Oui, maman.
-enfant-m|Je veux une feuille, moi aussi.
-maman|On regardera.
-narrateur|Ils prennent le sac.
-narrateur|La rue est calme.
-narrateur|En ce moment, Nino est à l'aire de jeux.
-narrateur|Le sable est un peu chaud.
-narrateur|Maman s'assoit au bord.
-narrateur|Nino a un seau vert.
-narrateur|Il a un manteau bleu posé au bord.
-narrateur|Il a son doudou ours.
-narrateur|Le petit toboggan est tiède.
-enfant-m|Il est chaud, maman.
+enfant-m|Elle danse !
+narrateur|Sur la vitre, un éclat de vitre cligne.
+maman|Tu vois l'éclat ?
+enfant-m|Il brille, sur le verre.
+narrateur|Maman pose la feuille sur le rebord.
+enfant-m|Je veux une feuille, maintenant !
+enfant-m|Dans mon seau vert !
+maman|On va à l'aire de jeux.
+narrateur|Ils prennent le sac, près de la porte.
+narrateur|La rue sent le sable chaud.
+narrateur|En ce moment, Nino pose le seau vert au bac.
+narrateur|Le sable est tiède, un peu collant.
+narrateur|Maman s'assoit au bord, à sa hauteur.
+narrateur|Le bac du toboggan tiède sent le sable.
+narrateur|Le manteau bleu attend au bord, plié.
+narrateur|L'ours doudou s'appuie au petit toboggan.
+enfant-m|Le toboggan est chaud.
 maman|Le soleil l'a touché.
 narrateur|Nino verse le sable.
-narrateur|Ça fait chh.
-narrateur|Une feuille passe.
-enfant-m|Une feuille, maman !
-maman|Comme celle de la fenêtre.
-maman|Elle danse.
-narrateur|La feuille se pose dans le seau.
-narrateur|Nino la sort tout doux.
-enfant-m|Elle habite ici.
-narrateur|Le vent reprend la feuille.
-narrateur|Elle s'envole au-dessus du bac.
-enfant-m|Elle est partie.
-maman|Elle vole encore.
+narrateur|Ça fait chh, dans le seau.
+narrateur|Une feuille orange passe, basse.
+enfant-m|La mienne, maintenant !
+narrateur|Elle se pose dans le seau vert.
+narrateur|Nino plaque la main dessus, vite.
+narrateur|Le seau bascule.
+narrateur|Du sable glisse, chaud.
+narrateur|La feuille s'envole au-dessus du bac.
+enfant-m|Elle est partie !
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Nino veut courir après la feuille.
+narrateur|Il tire le seau et le manteau, ensemble.
+narrateur|La manche se tord, à l'envers.
+narrateur|L'ours bascule, près du toboggan.
+enfant-m|Ça reste coincé !
 maman|C'est l'heure.
 enfant-m|La feuille aussi ?
 maman|La feuille peut voler.
-maman|Tes affaires viennent à la maison.
-maman|On reprend ses affaires, avant de partir.
+maman|Toi, tu reprends le seau ?
 narrateur|Nino cherche le seau.
-narrateur|Le seau est encore vert, un peu sableux.
+narrateur|Le seau est vert, un peu sableux.
 narrateur|Il le prend.
 enfant-m|J'ai le seau.
-maman|Bien.
-maman|On lui fera une place, à la maison.
 narrateur|Le manteau est au bord.
 narrateur|Une manche est à l'envers.
-narrateur|L'ours est près du toboggan.</t>
+narrateur|L'ours est près du toboggan.
+maman|Tu poses le seau un moment ?
+narrateur|Maman s'accroupit à sa hauteur.
+maman|Tu regardes tes affaires ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>fenetre,enfants_parc</t>
         </is>
       </c>
     </row>
@@ -1411,17 +1421,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Nino ?</t>
+          <t>Nino prépare le départ. Le seau, le manteau, l'ours attendent. Avant de partir, que fait Nino ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Nino ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nino prépare le départ. Le seau, le manteau, l'ours attendent. &lt;emphasis level="moderate"&gt;Avant de partir&lt;/emphasis&gt;, que fait Nino ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;&lt;emphasis&gt;avant&lt;/emphasis&gt; de partir, que fait Clément ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nino prépare le départ. Le seau, le manteau, l'ours attendent. &lt;emphasis&gt;Avant de partir&lt;/emphasis&gt;, que fait Nino ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1484,7 +1494,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1495,7 +1505,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1510,38 +1520,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>Avant de partir</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1556,22 +1566,24 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=avant_de_partir_il_reprend; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Avant de partir, que fait Nino ?</t>
+          <t>narrateur|Nino prépare le départ.
+narrateur|Le seau, le manteau, l'ours attendent.
+narrateur|Avant de partir, que fait Nino ?</t>
         </is>
       </c>
     </row>
@@ -1598,17 +1610,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nino cherche le manteau. Il tourne la manche tout doux. Le manteau est bleu. Il le prend. Et l'ours ? Nino va près du toboggan. L'ours est tiède, comme le plastique. L'ours est là. Il le prend. Tu as repris tes affaires. Avant de partir. Oui. La feuille de la fenêtre t'attend. Ils marchent vers la maison. Le seau cogne un peu. Le doudou est contre lui. Je marche à côté. Moi aussi.</t>
+          <t>Nino refuse de tirer plus fort. Il pose le seau vert, net. Je pose le seau. Nino reprend le manteau bleu. Il tourne la manche, lente. Le manteau est bleu. Il le passe, sans courir. Et l'ours ? Nino va près du toboggan. L'ours est tiède, comme le plastique. L'ours est là. Il reprend l'ours contre lui. Tu as tes affaires, Nino ? Oui, maman. Merci, Nino. On rentre vers la fenêtre ? Oui. Ils marchent vers la maison. Le seau cogne un peu, sableux. Contre lui, le doudou reste chaud. Je marche à côté. Moi aussi.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nino cherche le manteau. Il tourne la manche tout doux. Le manteau est bleu. Il le prend. Et l'ours ? Nino va près du toboggan. L'ours est tiède, comme le plastique. L'ours est là. Il le prend. Tu as repris tes affaires. Avant de partir. Oui. La feuille de la fenêtre t'attend. Ils marchent vers la maison. Le seau cogne un peu. Le doudou est contre lui. Je marche à côté. Moi aussi.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino refuse de tirer plus fort. Il pose le seau vert, net. Je pose le seau. Nino reprend le &lt;emphasis level="moderate"&gt;manteau&lt;/emphasis&gt; bleu. Il tourne la manche, lente. Le manteau est bleu. Il le passe, sans courir. Et l'ours ? Nino va près du toboggan. L'ours est tiède, comme le plastique. L'ours est là. Il reprend l'ours contre lui. Tu as tes affaires, Nino ? Oui, maman. Merci, Nino. On rentre vers la fenêtre ? Oui. Ils marchent vers la maison. Le seau cogne un peu, sableux. Contre lui, le doudou reste chaud. Je marche à côté. Moi aussi.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Clément a cherché. Il a repris le seau. Il a repris le manteau. Il a repris le doudou. C'était &lt;emphasis&gt;avant&lt;/emphasis&gt; de partir. [pause]</t>
+          <t>Nino refuse de tirer plus fort. Il pose le seau vert, net. Je pose le seau. Nino reprend le &lt;emphasis&gt;manteau&lt;/emphasis&gt; bleu. Il tourne la manche, lente. Le manteau est bleu. Il le passe, sans courir. Et l'ours ? Nino va près du toboggan. L'ours est tiède, comme le plastique. L'ours est là. Il reprend l'ours contre lui. Tu as tes affaires, Nino ? Oui, maman. Merci, Nino. On rentre vers la fenêtre ? Oui. Ils marchent vers la maison. Le seau cogne un peu, sableux. Contre lui, le doudou reste chaud. Je marche à côté. Moi aussi. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1666,7 +1678,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1689,7 +1701,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>manteau</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1703,16 +1715,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1737,31 +1749,40 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=fierté_calme; intensite=1; destinataire=enfant; sous_texte=il_reprend_sans_foncer; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nino cherche le manteau.
-narrateur|Il tourne la manche tout doux.
+          <t>narrateur|Nino refuse de tirer plus fort.
+narrateur|Il pose le seau vert, net.
+enfant-m|Je pose le seau.
+narrateur|Nino reprend le manteau bleu.
+narrateur|Il tourne la manche, lente.
 enfant-m|Le manteau est bleu.
-narrateur|Il le prend.
+narrateur|Il le passe, sans courir.
 maman|Et l'ours ?
 narrateur|Nino va près du toboggan.
 narrateur|L'ours est tiède, comme le plastique.
 enfant-m|L'ours est là.
-narrateur|Il le prend.
-maman|Tu as repris tes affaires.
-enfant-m|Avant de partir.
-maman|Oui.
-maman|La feuille de la fenêtre t'attend.
+narrateur|Il reprend l'ours contre lui.
+maman|Tu as tes affaires, Nino ?
+enfant-m|Oui, maman.
+maman|Merci, Nino.
+maman|On rentre vers la fenêtre ?
+enfant-m|Oui.
 narrateur|Ils marchent vers la maison.
-narrateur|Le seau cogne un peu.
-narrateur|Le doudou est contre lui.
+narrateur|Le seau cogne un peu, sableux.
+narrateur|Contre lui, le doudou reste chaud.
 maman|Je marche à côté.
 enfant-m|Moi aussi.</t>
         </is>
       </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>manteau,porte</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1786,17 +1807,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nino tient le seau. Maman ouvre la porte. La feuille du rebord est encore là. Elle a attendu. Oui. Tu poses le seau près de la fenêtre ? Nino pose le seau sous le rebord. Il pose le manteau. L'ours reste dans son bras. On met la feuille dans le seau ? Oui. Elle visite. Maman glisse la feuille orange. Elle tapote le fond. Toc. Elle danse plus. Ici, elle se repose. Bravo. Tu as repris tes affaires. La vitre est calme. Plus de toc, toc. L'ours regarde le seau.</t>
+          <t>Nino tient le seau, devant la porte. Maman ouvre. La feuille du rebord est là, orange. Elle a attendu ! Dans le seau, maintenant ! Il penche le seau trop vite. Du sable saute sur le rebord. La feuille bascule vers la fenêtre ouverte. Elle va partir ! Nino veut la rattraper d'un coup. Il refuse de foncer. Attends, je regarde. Maman attend, sans parler. Il observe le seau, puis la vitre. Sur le verre, un éclat de vitre cligne. C'est celui du début. Tu le vois, à la fenêtre ? Oui, il est resté. Nino pose le seau sous le rebord, lent. Il glisse la feuille orange, sans brusquer. Elle tapote le fond. Toc. Elle visite. Tu poses le manteau ? Nino pose le manteau près de la porte. L'ours reste dans son bras. La fenêtre se ferme un peu.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nino tient le seau. Maman ouvre la porte. La feuille du rebord est encore là. Elle a attendu. Oui. Tu poses le seau près de la fenêtre ? Nino pose le seau sous le rebord. Il pose le manteau. L'ours reste dans son bras. On met la feuille dans le seau ? Oui. Elle visite. Maman glisse la feuille orange. Elle tapote le fond. Toc. Elle danse plus. Ici, elle se repose. Bravo. Tu as repris tes affaires. La vitre est calme. Plus de toc, toc. L'ours regarde le seau.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nino tient le seau, devant la porte. Maman ouvre. La feuille du rebord est là, orange. Elle a attendu ! Dans le seau, maintenant ! Il penche le seau trop vite. Du sable saute sur le rebord. La feuille bascule vers la fenêtre ouverte. Elle va partir ! Nino veut la rattraper d'un coup. Il refuse de foncer. Attends, je regarde. Maman attend, sans parler. Il observe le seau, puis la vitre. Sur le verre, un &lt;emphasis level="moderate"&gt;éclat de vitre&lt;/emphasis&gt; cligne. C'est celui du début. Tu le vois, à la fenêtre ? Oui, il est resté. Nino pose le seau sous le rebord, lent. Il glisse la feuille orange, sans brusquer. Elle tapote le fond. Toc. Elle visite. Tu poses le manteau ? Nino pose le manteau près de la porte. L'ours reste dans son bras. La fenêtre se ferme un peu.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Clément tient le seau. Maman ouvre la porte. [pause]</t>
+          <t>&lt;low-pitch&gt;Nino tient le seau, devant la porte. Maman ouvre. La feuille du rebord est là, orange. Elle a attendu ! Dans le seau, maintenant ! Il penche le seau trop vite. Du sable saute sur le rebord. La feuille bascule vers la fenêtre ouverte. Elle va partir ! Nino veut la rattraper d'un coup. Il refuse de foncer. Attends, je regarde. Maman attend, sans parler. Il observe le seau, puis la vitre. Sur le verre, un &lt;emphasis&gt;éclat de vitre&lt;/emphasis&gt; cligne. C'est celui du début. Tu le vois, à la fenêtre ? Oui, il est resté. Nino pose le seau sous le rebord, lent. Il glisse la feuille orange, sans brusquer. Elle tapote le fond. Toc. Elle visite. Tu poses le manteau ? Nino pose le manteau près de la porte. L'ours reste dans son bras. La fenêtre se ferme un peu.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1843,7 +1864,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1851,22 +1872,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
         <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1875,28 +1900,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de vitre</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1905,45 +1934,59 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nino tient le seau.
-narrateur|Maman ouvre la porte.
-narrateur|La feuille du rebord est encore là.
-enfant-m|Elle a attendu.
-maman|Oui.
-maman|Tu poses le seau près de la fenêtre ?
-narrateur|Nino pose le seau sous le rebord.
-narrateur|Il pose le manteau.
-narrateur|L'ours reste dans son bras.
-maman|On met la feuille dans le seau ?
-enfant-m|Oui.
-enfant-m|Elle visite.
-narrateur|Maman glisse la feuille orange.
+          <t>narrateur|Nino tient le seau, devant la porte.
+narrateur|Maman ouvre.
+narrateur|La feuille du rebord est là, orange.
+enfant-m|Elle a attendu !
+enfant-m|Dans le seau, maintenant !
+narrateur|Il penche le seau trop vite.
+narrateur|Du sable saute sur le rebord.
+narrateur|La feuille bascule vers la fenêtre ouverte.
+enfant-m|Elle va partir !
+narrateur|Nino veut la rattraper d'un coup.
+narrateur|Il refuse de foncer.
+enfant-m|Attends, je regarde.
+narrateur|Maman attend, sans parler.
+narrateur|Il observe le seau, puis la vitre.
+narrateur|Sur le verre, un éclat de vitre cligne.
+enfant-m|C'est celui du début.
+maman|Tu le vois, à la fenêtre ?
+enfant-m|Oui, il est resté.
+narrateur|Nino pose le seau sous le rebord, lent.
+narrateur|Il glisse la feuille orange, sans brusquer.
 narrateur|Elle tapote le fond.
 narrateur|Toc.
-enfant-m|Elle danse plus.
-maman|Ici, elle se repose.
-maman|Bravo.
-maman|Tu as repris tes affaires.
-narrateur|La vitre est calme.
-narrateur|Plus de toc, toc.
-narrateur|L'ours regarde le seau.</t>
+enfant-m|Elle visite.
+maman|Tu poses le manteau ?
+narrateur|Nino pose le manteau près de la porte.
+narrateur|L'ours reste dans son bras.
+narrateur|La fenêtre se ferme un peu.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>porte</t>
         </is>
       </c>
     </row>
@@ -1970,17 +2013,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La feuille a sa place. Et toi, tu as repris tes affaires. Le seau vert reste sous la fenêtre.</t>
+          <t>La feuille a sa place. Le seau vert reste sous la fenêtre. Nino raccroche le manteau. Il est à sa place. Tu as fini de poser tes chaussures ? Oui, maman. La trace tiède de la paume a disparu. L'éclat de vitre reste, pâle, sur le verre. L'ours regarde le seau.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La feuille a sa place. Et toi, tu as repris tes affaires. Le seau vert reste sous la fenêtre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;La feuille a sa place. Le seau vert reste sous la fenêtre. Nino raccroche le manteau. Il est à sa place. Tu as fini de poser tes chaussures ? Oui, maman. La trace tiède de la paume a disparu. L'&lt;emphasis level="moderate"&gt;éclat de vitre&lt;/emphasis&gt; reste, pâle, sur le verre. L'ours regarde le seau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;La feuille a sa place. Le seau vert reste sous la fenêtre. Nino raccroche le manteau. Il est à sa place. Tu as fini de poser tes chaussures ? Oui, maman. La trace tiède de la paume a disparu. L'&lt;emphasis&gt;éclat de vitre&lt;/emphasis&gt; reste, pâle, sur le verre. L'ours regarde le seau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2027,7 +2070,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2035,10 +2078,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2047,12 +2090,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2061,17 +2104,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de vitre</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2080,11 +2127,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2093,26 +2140,41 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_reste_pale_le_seau_sous_la_fenetre; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
           <t>enfant-m|La feuille a sa place.
-maman|Et toi, tu as repris tes affaires.
-narrateur|Le seau vert reste sous la fenêtre.</t>
+narrateur|Le seau vert reste sous la fenêtre.
+narrateur|Nino raccroche le manteau.
+enfant-m|Il est à sa place.
+maman|Tu as fini de poser tes chaussures ?
+enfant-m|Oui, maman.
+narrateur|La trace tiède de la paume a disparu.
+narrateur|L'éclat de vitre reste, pâle, sur le verre.
+narrateur|L'ours regarde le seau.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>porte</t>
         </is>
       </c>
     </row>
@@ -2133,7 +2195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2225,6 +2287,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>